<commit_message>
US-15753 [IMP] Pick: Added 'display cancelled lines' to the lines filter. OUT: Added similar lines filter as the Pick. Removed Asset from PDF/XLSX/JSON export and imports, added 'Qty in Stock' in the exports
Signed-off-by: Dorian Kemps <dk@tempo-consulting.fr>
</commit_message>
<xml_diff>
--- a/bin/addons/msf_supply_doc_export/report/report_out_export.xlsx
+++ b/bin/addons/msf_supply_doc_export/report/report_out_export.xlsx
@@ -5,7 +5,7 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\192.168.123.1\partage1\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\192.168.122.1\partage1\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -117,9 +117,6 @@
     <t>BASE</t>
   </si>
   <si>
-    <t>Asset</t>
-  </si>
-  <si>
     <t>20 Deliver Unit</t>
   </si>
   <si>
@@ -160,6 +157,9 @@
   </si>
   <si>
     <t>PCE</t>
+  </si>
+  <si>
+    <t>Qty in Stock</t>
   </si>
 </sst>
 </file>
@@ -1052,11 +1052,10 @@
     <col min="1" max="1" width="18.140625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="36.42578125" bestFit="1" customWidth="1"/>
     <col min="3" max="4" width="45.42578125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="15.5703125" customWidth="1"/>
-    <col min="6" max="6" width="13.140625" customWidth="1"/>
-    <col min="7" max="7" width="14.5703125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="14.5703125" customWidth="1"/>
-    <col min="9" max="9" width="10.85546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.140625" customWidth="1"/>
+    <col min="6" max="6" width="14.5703125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14.5703125" customWidth="1"/>
+    <col min="8" max="9" width="10.85546875" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="13.42578125" customWidth="1"/>
     <col min="11" max="11" width="10.85546875" customWidth="1"/>
     <col min="12" max="13" width="10.85546875" bestFit="1" customWidth="1"/>
@@ -1117,7 +1116,7 @@
     </row>
     <row r="6" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B6" s="7" t="s">
         <v>4</v>
@@ -1131,7 +1130,7 @@
         <v>29</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C7" s="8">
         <v>3155690334</v>
@@ -1139,10 +1138,10 @@
     </row>
     <row r="8" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="B8" s="7" t="s">
         <v>34</v>
-      </c>
-      <c r="B8" s="7" t="s">
-        <v>35</v>
       </c>
     </row>
     <row r="9" spans="1:16" x14ac:dyDescent="0.25">
@@ -1167,22 +1166,22 @@
         <v>9</v>
       </c>
       <c r="E10" s="4" t="s">
-        <v>32</v>
+        <v>39</v>
       </c>
       <c r="F10" s="4" t="s">
-        <v>40</v>
+        <v>10</v>
       </c>
       <c r="G10" s="4" t="s">
-        <v>10</v>
+        <v>36</v>
       </c>
       <c r="H10" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="I10" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="J10" s="4" t="s">
         <v>37</v>
-      </c>
-      <c r="I10" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="J10" s="4" t="s">
-        <v>38</v>
       </c>
       <c r="K10" s="4" t="s">
         <v>30</v>
@@ -1194,13 +1193,13 @@
         <v>12</v>
       </c>
       <c r="N10" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="O10" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="O10" s="1" t="s">
+      <c r="P10" s="1" t="s">
         <v>42</v>
-      </c>
-      <c r="P10" s="1" t="s">
-        <v>43</v>
       </c>
     </row>
     <row r="11" spans="1:16" ht="30" x14ac:dyDescent="0.25">
@@ -1217,12 +1216,14 @@
         <v>16</v>
       </c>
       <c r="E11" s="7"/>
-      <c r="F11" s="7"/>
+      <c r="F11" s="7" t="s">
+        <v>13</v>
+      </c>
       <c r="G11" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="H11" s="7" t="s">
         <v>31</v>
+      </c>
+      <c r="H11" s="7">
+        <v>1</v>
       </c>
       <c r="I11" s="7">
         <v>1</v>
@@ -1231,7 +1232,7 @@
         <v>0</v>
       </c>
       <c r="K11" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="L11" s="7" t="s">
         <v>3</v>
@@ -1254,21 +1255,23 @@
         <v>5</v>
       </c>
       <c r="B12" s="7" t="s">
+        <v>43</v>
+      </c>
+      <c r="C12" s="7" t="s">
         <v>44</v>
-      </c>
-      <c r="C12" s="7" t="s">
-        <v>45</v>
       </c>
       <c r="D12" s="7" t="s">
         <v>17</v>
       </c>
       <c r="E12" s="7"/>
-      <c r="F12" s="7"/>
+      <c r="F12" s="7" t="s">
+        <v>13</v>
+      </c>
       <c r="G12" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="H12" s="7" t="s">
         <v>31</v>
+      </c>
+      <c r="H12" s="7">
+        <v>1</v>
       </c>
       <c r="I12" s="7">
         <v>1</v>
@@ -1277,7 +1280,7 @@
         <v>0</v>
       </c>
       <c r="K12" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="L12" s="7">
         <v>12345</v>

</xml_diff>